<commit_message>
Fix: separate recruit_type and startup_stage columns in ScoreReview; add pres_order sort in evaluator; parallel data loading
</commit_message>
<xml_diff>
--- a/기업명단_샘플.xlsx
+++ b/기업명단_샘플.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sensm\Desktop\12_기타문서\startup-recruitment-evaluation-system-pt\sample-data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SDY\Desktop\AI\evaluation-system-pt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD63576C-DDBA-4B1C-A8BB-D169231DD09F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{826AF643-877E-4D4F-84CA-35966D1263E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
   </definedNames>
   <calcPr calcId="0"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId4"/>
+    <pivotCache cacheId="2" r:id="rId4"/>
   </pivotCaches>
 </workbook>
 </file>
@@ -2156,58 +2156,58 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>공예ㆍ디자인-1</t>
-  </si>
-  <si>
-    <t>기계ㆍ소재-1</t>
-  </si>
-  <si>
-    <t>바이오ㆍ의료ㆍ생명-1</t>
-  </si>
-  <si>
-    <t>에너지ㆍ자원-1</t>
-  </si>
-  <si>
-    <t>전기ㆍ전자-1</t>
-  </si>
-  <si>
-    <t>정보ㆍ통신-1</t>
-  </si>
-  <si>
-    <t>화공ㆍ섬유-1</t>
-  </si>
-  <si>
-    <t>정보ㆍ통신-2</t>
-  </si>
-  <si>
-    <t>정보ㆍ통신-3</t>
-  </si>
-  <si>
-    <t>바이오ㆍ의료ㆍ생명-2</t>
-  </si>
-  <si>
-    <t>정보ㆍ통신-4</t>
-  </si>
-  <si>
-    <t>바이오ㆍ의료ㆍ생명-3</t>
-  </si>
-  <si>
-    <t>바이오ㆍ의료ㆍ생명-4</t>
-  </si>
-  <si>
-    <t>정보ㆍ통신-5</t>
-  </si>
-  <si>
-    <t>정보ㆍ통신-6</t>
-  </si>
-  <si>
-    <t>정보ㆍ통신-7</t>
-  </si>
-  <si>
-    <t>정보ㆍ통신-8</t>
-  </si>
-  <si>
-    <t>정보ㆍ통신-9</t>
+    <t>공예ㆍ디자인 1</t>
+  </si>
+  <si>
+    <t>기계ㆍ소재 1</t>
+  </si>
+  <si>
+    <t>바이오ㆍ의료ㆍ생명 1</t>
+  </si>
+  <si>
+    <t>에너지ㆍ자원 1</t>
+  </si>
+  <si>
+    <t>전기ㆍ전자 1</t>
+  </si>
+  <si>
+    <t>정보ㆍ통신 1</t>
+  </si>
+  <si>
+    <t>화공ㆍ섬유 1</t>
+  </si>
+  <si>
+    <t>정보ㆍ통신 2</t>
+  </si>
+  <si>
+    <t>정보ㆍ통신 3</t>
+  </si>
+  <si>
+    <t>바이오ㆍ의료ㆍ생명 2</t>
+  </si>
+  <si>
+    <t>정보ㆍ통신 4</t>
+  </si>
+  <si>
+    <t>바이오ㆍ의료ㆍ생명 3</t>
+  </si>
+  <si>
+    <t>바이오ㆍ의료ㆍ생명 4</t>
+  </si>
+  <si>
+    <t>정보ㆍ통신 5</t>
+  </si>
+  <si>
+    <t>정보ㆍ통신 6</t>
+  </si>
+  <si>
+    <t>정보ㆍ통신 7</t>
+  </si>
+  <si>
+    <t>정보ㆍ통신 8</t>
+  </si>
+  <si>
+    <t>정보ㆍ통신 9</t>
   </si>
 </sst>
 </file>
@@ -2258,7 +2258,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="표준" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4">
@@ -7205,7 +7205,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{12BEC9E0-B3D4-4F2D-87E8-3DF9422899BB}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{12BEC9E0-B3D4-4F2D-87E8-3DF9422899BB}" name="PivotTable1" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:B12" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="20">
     <pivotField showAll="0"/>

</xml_diff>